<commit_message>
Update training data and HR drift analysis
</commit_message>
<xml_diff>
--- a/data/training_plan.xlsx
+++ b/data/training_plan.xlsx
@@ -5,41 +5,22 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hilton-my.sharepoint.com/personal/koen_klinkenberg_hilton_com/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kklinkenberg1\garmin-training-analysis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="234" documentId="8_{42B50EE8-AFFA-4B9A-854C-7437D9BC5F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0171BEB-80A3-4812-8D03-49602109AA71}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C00AF6BC-D4F2-4C01-98F1-0DBB426B9BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C3605B99-7A81-41CA-BE46-834C8704C4BE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planned Sessions" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="75">
   <si>
     <t>Date</t>
   </si>
@@ -50,13 +31,16 @@
     <t>Sport</t>
   </si>
   <si>
+    <t>Planned Distance (km)</t>
+  </si>
+  <si>
+    <t>Planned Time (min)</t>
+  </si>
+  <si>
     <t>Notes</t>
   </si>
   <si>
-    <t>Planned Distance (km)</t>
-  </si>
-  <si>
-    <t>Planned Time (min)</t>
+    <t>Recovery Swim</t>
   </si>
   <si>
     <t>Swimming</t>
@@ -74,84 +58,84 @@
     <t>Session A</t>
   </si>
   <si>
+    <t>Tempo Run</t>
+  </si>
+  <si>
     <t>Running</t>
   </si>
   <si>
     <t>2 km easy, then 3x8 minutes at controlled tempo/LT2 effort with 3 minutes easy jogging in between. Then cool down of 2-3 km. Effort not above 7/10</t>
   </si>
   <si>
+    <t>Easy Bike</t>
+  </si>
+  <si>
+    <t>Cycling</t>
+  </si>
+  <si>
+    <t>45-60</t>
+  </si>
+  <si>
+    <t>Very easy, shorter if fatigued</t>
+  </si>
+  <si>
+    <t>Easy Run</t>
+  </si>
+  <si>
+    <t>4x15 seonds strides if recovered</t>
+  </si>
+  <si>
+    <t>Session B, no plyo metrics</t>
+  </si>
+  <si>
+    <t>Technical Swim</t>
+  </si>
+  <si>
+    <t>45-55</t>
+  </si>
+  <si>
+    <t>Include repititions but focus on technique</t>
+  </si>
+  <si>
+    <t>Aerobic Bike</t>
+  </si>
+  <si>
+    <t>75-90</t>
+  </si>
+  <si>
+    <t>3x6 at 150-160 bpm with 4 minutes recovery, rest 135-150 bpm</t>
+  </si>
+  <si>
+    <t>Recovery Run</t>
+  </si>
+  <si>
+    <t>Very easy, Z1</t>
+  </si>
+  <si>
+    <t>Easy, 145-155 bpm</t>
+  </si>
+  <si>
+    <t>Long Run</t>
+  </si>
+  <si>
+    <t>First 12 km easy, not above 155-158. Last 3 km sits close to LT! (163 bpm)</t>
+  </si>
+  <si>
+    <t>35-45</t>
+  </si>
+  <si>
     <t>Easy</t>
   </si>
   <si>
-    <t>Cycling</t>
-  </si>
-  <si>
-    <t>45-60</t>
-  </si>
-  <si>
-    <t>Very easy, shorter if fatigued</t>
-  </si>
-  <si>
-    <t>45-55</t>
-  </si>
-  <si>
-    <t>Include repititions but focus on technique</t>
-  </si>
-  <si>
-    <t>75-90</t>
-  </si>
-  <si>
-    <t>4x15 seonds strides if recovered</t>
-  </si>
-  <si>
-    <t>Session B, no plyo metrics</t>
-  </si>
-  <si>
-    <t>Long Run</t>
-  </si>
-  <si>
-    <t>Easy Run</t>
-  </si>
-  <si>
-    <t>Tempo Run</t>
-  </si>
-  <si>
-    <t>Very easy, Z1</t>
-  </si>
-  <si>
-    <t>Easy, 145-155 bpm</t>
-  </si>
-  <si>
-    <t>Recovery Swim</t>
-  </si>
-  <si>
-    <t>Recovery Run</t>
-  </si>
-  <si>
-    <t>Technical Swim</t>
-  </si>
-  <si>
-    <t>35-45</t>
-  </si>
-  <si>
     <t>Session A, plyo can be included</t>
   </si>
   <si>
     <t>Threshold 1 Run</t>
   </si>
   <si>
-    <t>First 12 km easy, not above 155-158. Last 3 km sits close to LT! (163 bpm)</t>
-  </si>
-  <si>
     <t>2km easy, 6 km continuous LT1, 3 km easy. Objective is stable HR, meaning if HR keeps rising, pace needs to come down.</t>
   </si>
   <si>
-    <t>Easy Bike</t>
-  </si>
-  <si>
-    <t>Aerobic Bike</t>
-  </si>
-  <si>
     <t>Recovery effort</t>
   </si>
   <si>
@@ -170,9 +154,6 @@
     <t>6x30 seconds high cadence, rest 135-150 bpm</t>
   </si>
   <si>
-    <t>3x6 at 150-160 bpm with 4 minutes recovery, rest 135-150 bpm</t>
-  </si>
-  <si>
     <t>RPE 2-3/10. Slow enough to protect volleyball practice</t>
   </si>
   <si>
@@ -218,18 +199,18 @@
     <t>Light, calf, soleus, glute, core, shore. No heavy sets</t>
   </si>
   <si>
+    <t>25-40</t>
+  </si>
+  <si>
+    <t>Relaxed</t>
+  </si>
+  <si>
     <t>40-50</t>
   </si>
   <si>
     <t>Easy spinning</t>
   </si>
   <si>
-    <t>25-40</t>
-  </si>
-  <si>
-    <t>Relaxed</t>
-  </si>
-  <si>
     <t>Very easy (140-150 bpm)</t>
   </si>
   <si>
@@ -243,6 +224,27 @@
   </si>
   <si>
     <t>Controlled, executon as planned</t>
+  </si>
+  <si>
+    <t>0-12</t>
+  </si>
+  <si>
+    <t>12-15:Controlled</t>
+  </si>
+  <si>
+    <t>12-16:Controlled;16-17:Recovery</t>
+  </si>
+  <si>
+    <t>0-4</t>
+  </si>
+  <si>
+    <t>4-5:Fast Finish</t>
+  </si>
+  <si>
+    <t>Drift Segment</t>
+  </si>
+  <si>
+    <t>Work Segment</t>
   </si>
 </sst>
 </file>
@@ -312,7 +314,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>505661</xdr:colOff>
+      <xdr:colOff>512012</xdr:colOff>
       <xdr:row>94</xdr:row>
       <xdr:rowOff>172229</xdr:rowOff>
     </xdr:to>
@@ -321,7 +323,7 @@
         <xdr:cNvPr id="6" name="Picture 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5EF8CB22-7650-7DA5-4CD4-116538E946CE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -343,6 +345,9 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -356,7 +361,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>26</xdr:col>
-      <xdr:colOff>486877</xdr:colOff>
+      <xdr:colOff>493228</xdr:colOff>
       <xdr:row>103</xdr:row>
       <xdr:rowOff>39149</xdr:rowOff>
     </xdr:to>
@@ -365,7 +370,7 @@
         <xdr:cNvPr id="9" name="Picture 8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F84AAEEE-295F-844F-D74E-1A4A29153665}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -387,6 +392,9 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -400,16 +408,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>26</xdr:col>
-      <xdr:colOff>372560</xdr:colOff>
+      <xdr:colOff>378911</xdr:colOff>
       <xdr:row>143</xdr:row>
-      <xdr:rowOff>67725</xdr:rowOff>
+      <xdr:rowOff>74075</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="10" name="Picture 9">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{36F04BC9-39B3-8553-5F4F-5DDF0C87F2B8}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000A000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -431,6 +439,9 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -754,19 +765,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF0A92FC-49B4-40DA-A35E-FB06DEA176B7}">
-  <dimension ref="A1:F34"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="147" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="154" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -777,52 +790,58 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>46293</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>46293</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>46294</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D4">
         <v>10</v>
@@ -831,35 +850,35 @@
         <v>50</v>
       </c>
       <c r="F4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>46294</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>46295</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D6">
         <v>7</v>
@@ -868,52 +887,52 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>46295</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>46296</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E8" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>46296</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="C9" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E9" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>46297</v>
       </c>
@@ -921,171 +940,183 @@
         <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D10">
         <v>5</v>
       </c>
       <c r="F10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>46298</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D11">
         <v>4</v>
       </c>
       <c r="F11" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+      <c r="G11" t="s">
+        <v>71</v>
+      </c>
+      <c r="H11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>46299</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D12">
         <v>15</v>
       </c>
       <c r="F12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+      <c r="G12" t="s">
+        <v>68</v>
+      </c>
+      <c r="H12" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>46300</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E13" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>46300</v>
       </c>
       <c r="C14" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F14" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>46301</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C15" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D15">
         <v>11</v>
       </c>
       <c r="F15" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>46301</v>
       </c>
       <c r="B16" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E16" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F16" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>46302</v>
       </c>
       <c r="B17" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C17" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D17">
         <v>8</v>
       </c>
       <c r="F17" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>46302</v>
       </c>
       <c r="C18" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>46303</v>
       </c>
       <c r="C19" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E19" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F19" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>46303</v>
       </c>
       <c r="B20" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="C20" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E20" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F20" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>46304</v>
       </c>
@@ -1093,7 +1124,7 @@
         <v>28</v>
       </c>
       <c r="C21" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D21">
         <v>6</v>
@@ -1102,41 +1133,47 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>46305</v>
       </c>
       <c r="B22" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C22" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D22">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="F22" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+        <v>46</v>
+      </c>
+      <c r="G22" t="s">
+        <v>68</v>
+      </c>
+      <c r="H22" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>46306</v>
       </c>
       <c r="B23" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C23" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D23">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="F23" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>46307</v>
       </c>
@@ -1144,7 +1181,7 @@
         <v>47</v>
       </c>
       <c r="C24" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E24" t="s">
         <v>48</v>
@@ -1153,12 +1190,12 @@
         <v>49</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>46307</v>
       </c>
       <c r="C25" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E25" t="s">
         <v>48</v>
@@ -1167,7 +1204,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>46308</v>
       </c>
@@ -1175,7 +1212,7 @@
         <v>51</v>
       </c>
       <c r="C26" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E26" t="s">
         <v>52</v>
@@ -1184,7 +1221,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
         <v>46308</v>
       </c>
@@ -1192,7 +1229,7 @@
         <v>54</v>
       </c>
       <c r="C27" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E27" t="s">
         <v>55</v>
@@ -1201,15 +1238,15 @@
         <v>56</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
         <v>46309</v>
       </c>
       <c r="B28" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C28" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D28">
         <v>5</v>
@@ -1218,12 +1255,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
         <v>46309</v>
       </c>
       <c r="C29" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E29" t="s">
         <v>57</v>
@@ -1232,49 +1269,49 @@
         <v>58</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
         <v>46310</v>
       </c>
       <c r="B30" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="C30" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E30" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F30" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
         <v>46310</v>
       </c>
       <c r="B31" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="C31" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E31" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F31" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
         <v>46311</v>
       </c>
       <c r="B32" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C32" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D32">
         <v>3</v>
@@ -1291,7 +1328,7 @@
         <v>64</v>
       </c>
       <c r="C33" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D33">
         <v>2</v>
@@ -1308,7 +1345,7 @@
         <v>66</v>
       </c>
       <c r="C34" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D34">
         <v>21.1</v>

</xml_diff>